<commit_message>
Track manuscript revision 6a9dfe7: complete-cases RQ3 (n = 59)
The co-authors adopted the exclusion of the partial security responder
(P53), matching their v2.1 scripts and the September notebooks. Security
scores are now defined only for complete six-item responses; RQ3 and the
correlations run on n = 59; the analysis adds the paper's new post-hoc
per-treatment benchmark tests (t, LCB, Wilcoxon, sign, Holm), the TOST
equivalence at d-based margins, and the Fisher-Freeman-Halton exact
attrition tests by treatment and day. The notebooks are refreshed from
reproduction/v2 (security_perception, security_boxplot, updated Spearman)
and paper_values.json now tracks the current manuscript: 103 of 104
values reproduce; the one exception is the T2 correlation misprint
(computed 0.817, printed 0.81).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFB9D3TRc1CNMH2d7VooMa
</commit_message>
<xml_diff>
--- a/output/notebooks/resumen_tratamientos_seguridad.xlsx
+++ b/output/notebooks/resumen_tratamientos_seguridad.xlsx
@@ -485,16 +485,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>35.89</v>
+        <v>37.5</v>
       </c>
       <c r="D3" t="n">
         <v>37.5</v>
       </c>
       <c r="E3" t="n">
-        <v>12.88</v>
+        <v>11.86</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>39.92</v>
+        <v>40.73</v>
       </c>
       <c r="D7" t="n">
-        <v>41.25</v>
+        <v>42.5</v>
       </c>
       <c r="E7" t="n">
-        <v>14.18</v>
+        <v>13.65</v>
       </c>
       <c r="F7" t="n">
         <v>10</v>

</xml_diff>